<commit_message>
Bug fixes and better error output
</commit_message>
<xml_diff>
--- a/SystemData/System_Specifications.xlsx
+++ b/SystemData/System_Specifications.xlsx
@@ -211,39 +211,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -586,13 +586,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="n">
-        <v>43.5777837731445</v>
+        <v>43.5</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>1.46054537382289</v>
+        <v>1.46</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>145.584930419922</v>
+        <v>145</v>
       </c>
       <c r="D2" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Show NASA warning if unavailable data
</commit_message>
<xml_diff>
--- a/SystemData/System_Specifications.xlsx
+++ b/SystemData/System_Specifications.xlsx
@@ -211,39 +211,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -586,13 +586,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="n">
-        <v>43.5</v>
+        <v>43.5777837731445</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>1.46</v>
+        <v>1.46054537382289</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>145</v>
+        <v>145.584930419922</v>
       </c>
       <c r="D2" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Fix multiple errors. Update SystemSpecificationx.xlsx column names.
</commit_message>
<xml_diff>
--- a/SystemData/System_Specifications.xlsx
+++ b/SystemData/System_Specifications.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -52,10 +52,10 @@
     <t xml:space="preserve">Calib square size (mm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Start year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End year</t>
+    <t xml:space="preserve">Start date (YYYYMMDD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">End date (YYYYMMDD)</t>
   </si>
   <si>
     <t xml:space="preserve">Solar panel peak wattage (W)</t>
@@ -211,39 +211,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -506,8 +506,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="19.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="20.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="17.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="16.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="21.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="27.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="24.29"/>

</xml_diff>